<commit_message>
Incorporated Nikki's requested changes in the email
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.00233073156143</v>
+        <v>0.9966779411813623</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.036901331631477</v>
+        <v>1.022535252892402</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.077127994947791</v>
+        <v>1.052206059847206</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.123939061743652</v>
+        <v>1.0918426735596</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.177276671102982</v>
+        <v>1.136897217591656</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.015673086120904</v>
+        <v>0.9754429137160815</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.085326006172266</v>
+        <v>1.033771105585218</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.165507499632763</v>
+        <v>1.097544767314922</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.245467929459578</v>
+        <v>1.170868364458936</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.327576367404846</v>
+        <v>1.245311863681312</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.418366206205416</v>
+        <v>1.318591226360277</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.176237334817857</v>
+        <v>1.114661133623676</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.208428663362028</v>
+        <v>1.136821334735611</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.297689579911427</v>
+        <v>1.212972828891542</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.26538102185564</v>
+        <v>1.164426957550531</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.315210554336267</v>
+        <v>1.238466547951887</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.33528225066841</v>
+        <v>1.269325931531725</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.388964826765446</v>
+        <v>1.348713573407885</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.266322499250806</v>
+        <v>1.245857705247396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed User input file to import data from Spreadsheet
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9966779411813623</v>
+        <v>1.001524187043356</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.022535252892402</v>
+        <v>1.035996632312221</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.052206059847206</v>
+        <v>1.082444383054403</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.0918426735596</v>
+        <v>1.135842614825424</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.136897217591656</v>
+        <v>1.194768468643236</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0.9754429137160815</v>
+        <v>1.025275377405232</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.033771105585218</v>
+        <v>1.096490980281946</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.097544767314922</v>
+        <v>1.17659068410322</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.170868364458936</v>
+        <v>1.259117251487194</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.245311863681312</v>
+        <v>1.343104746568216</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.318591226360277</v>
+        <v>1.427456452720722</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.114661133623676</v>
+        <v>1.182820957993607</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.136821334735611</v>
+        <v>1.198859872339649</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.212972828891542</v>
+        <v>1.286751956227349</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.164426957550531</v>
+        <v>1.248331902866396</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.238466547951887</v>
+        <v>1.297740613120589</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.269325931531725</v>
+        <v>1.316275351024059</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.348713573407885</v>
+        <v>1.367047533106612</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.245857705247396</v>
+        <v>1.241103685255613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated user inputs; updated config and utils files, vectorisd multiple iterations function; made all years in plots actual years
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.001524187043356</v>
+        <v>1.223190534761459</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.035996632312221</v>
+        <v>0.9814895949464031</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.082444383054403</v>
+        <v>1.016471858552005</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.135842614825424</v>
+        <v>1.05984713954409</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.194768468643236</v>
+        <v>1.109280203685029</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.025275377405232</v>
+        <v>1.16567161862703</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.096490980281946</v>
+        <v>1.203863546698453</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.17659068410322</v>
+        <v>1.109691253312778</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.259117251487194</v>
+        <v>1.116375371619652</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.343104746568216</v>
+        <v>1.153913925497934</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.427456452720722</v>
+        <v>1.130646402805523</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.182820957993607</v>
+        <v>1.171236210877145</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.198859872339649</v>
+        <v>1.189823307349178</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.286751956227349</v>
+        <v>1.236556455676249</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.248331902866396</v>
+        <v>1.141405111806231</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.297740613120589</v>
+        <v>1.108774782995134</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.316275351024059</v>
+        <v>1.160547834281969</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.367047533106612</v>
+        <v>1.21369588409696</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.241103685255613</v>
+        <v>1.266982840412876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added katyas updates to pcm from ds. model is running. 12.09.2025
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.080129928708779</v>
+        <v>1.078165243422068</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.10478420341286</v>
+        <v>1.10865408842026</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.132375031716253</v>
+        <v>1.14534186698654</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.159927413846156</v>
+        <v>1.178906447822625</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.187249469457665</v>
+        <v>1.213774147594684</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.214246140395895</v>
+        <v>1.247977008756527</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.240762328565538</v>
+        <v>1.281782333025806</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.267635819790895</v>
+        <v>1.315001846963764</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.294275456077319</v>
+        <v>1.347493858139045</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.319521670252862</v>
+        <v>1.379840470117618</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.345191879795006</v>
+        <v>1.411018229368153</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.370144040361042</v>
+        <v>1.442119703959621</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.394259086022622</v>
+        <v>1.472156254482162</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.417998137775826</v>
+        <v>1.501293693960544</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.44084418387691</v>
+        <v>1.529412256823917</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.462783200365625</v>
+        <v>1.557245058596096</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.4847070306661</v>
+        <v>1.583546177426379</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.506438682440474</v>
+        <v>1.609738559410429</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.527083474832873</v>
+        <v>1.634362265942956</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ds on pmc working. ss on gr function not working and not intergrated yet.
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.078165243422068</v>
+        <v>1.204542114739566</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.10865408842026</v>
+        <v>1.222402935862552</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.14534186698654</v>
+        <v>1.240654675983215</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.178906447822625</v>
+        <v>1.258905813743022</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.213774147594684</v>
+        <v>1.277048170199546</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.247977008756527</v>
+        <v>1.295663376935416</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.281782333025806</v>
+        <v>1.314227396891755</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.315001846963764</v>
+        <v>1.332399721743222</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.347493858139045</v>
+        <v>1.350703891707488</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.379840470117618</v>
+        <v>1.368444152933959</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.411018229368153</v>
+        <v>1.385829370414834</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.442119703959621</v>
+        <v>1.403544065638238</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.472156254482162</v>
+        <v>1.413604250174934</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.501293693960544</v>
+        <v>1.423876335321453</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.529412256823917</v>
+        <v>1.434123046789749</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.557245058596096</v>
+        <v>1.44411739422053</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.583546177426379</v>
+        <v>1.453926922280963</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.609738559410429</v>
+        <v>1.463536327550345</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.634362265942956</v>
+        <v>1.473416373610477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
model running -- indent issues fixed
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.204542114739566</v>
+        <v>1.202204608701802</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.222402935862552</v>
+        <v>1.217819708918407</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.240654675983215</v>
+        <v>1.23359280072673</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.258905813743022</v>
+        <v>1.249030938993507</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.277048170199546</v>
+        <v>1.264366297350701</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.295663376935416</v>
+        <v>1.279227254871736</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.314227396891755</v>
+        <v>1.294012050465161</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.332399721743222</v>
+        <v>1.308901799415134</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.350703891707488</v>
+        <v>1.323413038329474</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.368444152933959</v>
+        <v>1.337952440711086</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.385829370414834</v>
+        <v>1.351938516066043</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.403544065638238</v>
+        <v>1.360189373377525</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.413604250174934</v>
+        <v>1.368132440004313</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.423876335321453</v>
+        <v>1.375851443939394</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.434123046789749</v>
+        <v>1.383664916486916</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.44411739422053</v>
+        <v>1.391145174093756</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.453926922280963</v>
+        <v>1.39879212610556</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.463536327550345</v>
+        <v>1.406531178275171</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.473416373610477</v>
+        <v>1.414021853410145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
running with sediment exposure impacting growth rate - need to check outputs are correct
</commit_message>
<xml_diff>
--- a/output/Rugosity_growth_param_0.5.xlsx
+++ b/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.202204608701802</v>
+        <v>1.195559970613224</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.217819708918407</v>
+        <v>1.204283990132534</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.23359280072673</v>
+        <v>1.212876987385829</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.249030938993507</v>
+        <v>1.22100598048646</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.264366297350701</v>
+        <v>1.228343577575312</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.279227254871736</v>
+        <v>1.235982368673371</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.294012050465161</v>
+        <v>1.24262230340046</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.308901799415134</v>
+        <v>1.249472196929326</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.323413038329474</v>
+        <v>1.255902278324754</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.337952440711086</v>
+        <v>1.259469442984582</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.351938516066043</v>
+        <v>1.262922154656091</v>
       </c>
     </row>
     <row r="14">
@@ -536,7 +536,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>1.360189373377525</v>
+        <v>1.266176791455366</v>
       </c>
     </row>
     <row r="15">
@@ -544,7 +544,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>1.368132440004313</v>
+        <v>1.269081277320885</v>
       </c>
     </row>
     <row r="16">
@@ -552,7 +552,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>1.375851443939394</v>
+        <v>1.271916717848958</v>
       </c>
     </row>
     <row r="17">
@@ -560,7 +560,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>1.383664916486916</v>
+        <v>1.274517277912264</v>
       </c>
     </row>
     <row r="18">
@@ -568,7 +568,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>1.391145174093756</v>
+        <v>1.276787320341926</v>
       </c>
     </row>
     <row r="19">
@@ -576,7 +576,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>1.39879212610556</v>
+        <v>1.278531434915943</v>
       </c>
     </row>
     <row r="20">
@@ -584,7 +584,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>1.406531178275171</v>
+        <v>1.280210191261991</v>
       </c>
     </row>
     <row r="21">
@@ -592,7 +592,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>1.414021853410145</v>
+        <v>1.281953309008222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>